<commit_message>
docs(competitors): yellow-highlight every cell the 14 September response update touched
45 cells: the changed Compliance Level / Description / Non-Compliance cells of
the 30 re-answered user stories, and the dated line on the Vision sheet. One
solid-yellow fill added to styles.xml and the two affected cell styles cloned
with it, so fonts, borders and wrapping are unchanged.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/competitors/BPM Tool Functional Requirements - Diagramatix.xlsx
+++ b/competitors/BPM Tool Functional Requirements - Diagramatix.xlsx
@@ -1674,7 +1674,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1738,6 +1738,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1829,7 +1835,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1941,6 +1947,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2266,7 +2278,7 @@
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B10" s="32" t="inlineStr">
+      <c r="B10" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagramatix response — updated 14 September 2026 (product 2.11, 165 user stories across 19 FR domains). Earlier revisions: 8 July 2026, 5 July 2026.</t>
         </is>
@@ -2784,7 +2796,7 @@
           <t xml:space="preserve">Comply with 3rd party Module</t>
         </is>
       </c>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagramatix exports BPMN 2.0 XML that executable workflow engines (e.g. Camunda, Flowable, Azure Logic Apps) consume to run workflows from the published process. The .bpmn export carries default flows and BPSim parameters and round-trips.</t>
         </is>
@@ -2811,17 +2823,17 @@
       <c r="E4" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="F4" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comply</t>
-        </is>
-      </c>
-      <c r="G4" s="39" t="inlineStr">
+      <c r="F4" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
+        </is>
+      </c>
+      <c r="G4" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagramatix Miner monitors executing workflows from their event data: live connectors (webhook push and on-demand refresh) keep a log current; linked run series follow the same process over time; period comparison refuses to compare two runs that are not the same process; and alerts lead with the one nobody else leads with — the source stopped sending. Case-level deviation evidence and hand-off / rework analysis explain what changed.</t>
         </is>
       </c>
-      <c r="H4" s="39"/>
+      <c r="H4" s="43"/>
     </row>
     <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
@@ -3760,7 +3772,7 @@
           <t xml:space="preserve">Partially Comply</t>
         </is>
       </c>
-      <c r="G9" s="39" t="inlineStr">
+      <c r="G9" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">The Risk-Control Matrix, Control Register, GRC Register, traceability graph and coverage summary all export to a multi-sheet Excel workbook in the format auditors expect. APQC coverage analytics additionally report which standard processes are modelled versus gaps, by category and level. Mining analyses and simulation business cases export to Excel / Word / PDF, and the Process API returns pools, lanes and an ordered activity list for a third party's own reporting.</t>
         </is>
@@ -3879,17 +3891,17 @@
       <c r="E13" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="F13" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comply</t>
-        </is>
-      </c>
-      <c r="G13" s="39" t="inlineStr">
+      <c r="F13" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
+        </is>
+      </c>
+      <c r="G13" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">The AI SOP generator produces a Standard Operating Procedure per role (lane), per pool, per sub-process or for the whole process — diagram-grounded (a deterministic extract, so it never invents steps), with each role's hand-offs (received-from / handed-off-to) and a cropped lane figure. Editable in-app, regenerated non-destructively, exported to Word adopting the organisation's Word template styles; each SOP records who generated it, when and with which model.</t>
         </is>
       </c>
-      <c r="H13" s="39"/>
+      <c r="H13" s="43"/>
     </row>
     <row r="14" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
@@ -3912,7 +3924,7 @@
           <t xml:space="preserve">Partially Comply</t>
         </is>
       </c>
-      <c r="G14" s="39" t="inlineStr">
+      <c r="G14" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Governance reporting includes a control-coverage summary, segregation-of-duties findings, per-control operating-effectiveness where mined, and a roll-up of control-effectiveness by APQC process category — all exportable to Excel for audit and compliance review. The SOP generator's step table lists role, task and the documents / data objects used per step, and the Diff report tabulates two versions side by side.</t>
         </is>
@@ -4154,7 +4166,7 @@
           <t xml:space="preserve">Partially Comply</t>
         </is>
       </c>
-      <c r="G5" s="39" t="inlineStr">
+      <c r="G5" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Processes are searchable/filterable by owner, author (modeller) and project; Business Unit/Group is represented via Entity Lists, and APQC PCF classification adds an industry-standard process-category facet. The project navigation tree filters by diagram type, name and feature badge (AI-generated, simulation, mining, APQC, risk &amp; control).</t>
         </is>
@@ -4753,17 +4765,17 @@
       <c r="E3" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="F3" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comply</t>
-        </is>
-      </c>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="F3" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
+        </is>
+      </c>
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Training material is generated from the models: role-based SOPs (Word) from the SOP generator, published process documentation, Visio / image / PDF exports for courseware, and Screencast Studio records narrated walk-throughs of a process directly in the tool (webm → mp4).</t>
         </is>
       </c>
-      <c r="H3" s="39"/>
+      <c r="H3" s="43"/>
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
@@ -4842,7 +4854,7 @@
           <t xml:space="preserve">Partially Comply</t>
         </is>
       </c>
-      <c r="G6" s="39" t="inlineStr">
+      <c r="G6" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Available guidance is surfaced via Bubble Help and the User Guide contextually. The User Guide opens at the chapter for the screen you are on and returns you to exactly where you left; Bubble Help annotates each control.</t>
         </is>
@@ -5944,7 +5956,7 @@
           <t xml:space="preserve">Partially Comply</t>
         </is>
       </c>
-      <c r="G8" s="39" t="inlineStr">
+      <c r="G8" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Configurable palettes and templates add reusable shapes to the modelling set. Icon Maintenance lets an administrator add custom icons / symbols to the ArchiMate library.</t>
         </is>
@@ -6390,7 +6402,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G4" s="39" t="inlineStr">
+      <c r="G4" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">The Simulator reports on runs with results, scenario comparison and Monte Carlo ranges. Beyond run results: a Welch significance test with a confidence interval, a parameter sweep with the knee marked, a sensitivity tornado (every input ±20%, ranked), validation of the simulated flow-time distribution against the real one (p50/p90/p95), suggested next steps from the run history, and a business case with a payback month exportable to Word / Excel / PDF.</t>
         </is>
@@ -6418,7 +6430,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G5" s="39" t="inlineStr">
+      <c r="G5" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Simulation data is provided via simulation parameters/calendars, and Diagramatix Miner calibrates it automatically from real event logs. Simulation Data lists what each diagram carries; lognormal and empirical distributions are selectable; skills held by people and required by tasks, and queue disciplines (FIFO, priority, shortest-job-first), are part of the input set.</t>
         </is>
@@ -6644,7 +6656,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagramatix Miner imports process-related event-log data (CSV/TSV, IEEE XES 1849 and OCEL 2.0/1.0) from the applications used in a process or set of processes. Excel workbooks (including wide 'one row per case' exports) and several systems' extracts merged into one lifecycle are imported in the import screen, and live connectors (webhook push, on-demand refresh) keep a log current.</t>
         </is>
@@ -6672,7 +6684,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G4" s="39" t="inlineStr">
+      <c r="G4" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagramatix Miner maps the extracted log columns (case, activity, timestamp, state, resource) to the Tasks/Activities and reference lifecycle in the model. A sparse log can be enriched from the project's own models.</t>
         </is>
@@ -6700,7 +6712,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G5" s="39" t="inlineStr">
+      <c r="G5" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagramatix Miner reports process performance and conformance from the extracted data, with an AI "Explain results" summary. Slicing with declared exactness, case-level deviation evidence ('fourteen cases skipped the credit check — here they are'), hand-off and rework analysis, elapsed-time attribution between steps, period comparison and alerting; analyses export to Excel.</t>
         </is>
@@ -6728,7 +6740,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G6" s="39" t="inlineStr">
+      <c r="G6" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagramatix Miner visualises performance by discovering the implied BPMN, overlaying conformance and calibrating a runnable simulation digital twin. Object-centric (OCEL) logs discover a domain model per object type.</t>
         </is>
@@ -7241,7 +7253,7 @@
           <t xml:space="preserve">Partially Comply</t>
         </is>
       </c>
-      <c r="G13" s="39" t="inlineStr">
+      <c r="G13" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagram history and Organisation Admin oversight show modelling activity and change history. The Registered Users console shows what each modeller is working on right now, and AI usage is metered per user.</t>
         </is>
@@ -7296,17 +7308,17 @@
       <c r="E15" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="F15" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comply</t>
-        </is>
-      </c>
-      <c r="G15" s="39" t="inlineStr">
+      <c r="F15" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
+        </is>
+      </c>
+      <c r="G15" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">A dedicated mobile view (/m) presents process models on phones and tablets — real colours, wrapped labels, sub-process/gateway/event/connector fidelity, rotate and pan-anywhere — and lets the reader add and save Review Comments from the device; desktop overlays are hidden. Browser-based, so nothing to install.</t>
         </is>
       </c>
-      <c r="H15" s="39"/>
+      <c r="H15" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8168,7 +8180,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G4" s="39" t="inlineStr">
+      <c r="G4" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagram feedback/comments gather improvement suggestions against any process. Per-element Pain Point / Issue markers and Review notes are available on every diagram type, and view-only recipients can drop notes that land in the owner's panel.</t>
         </is>
@@ -8463,7 +8475,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">ArchiMate modelling and cross-diagram drill-down relate business processes to capabilities and functions, and the APQC Process Classification Framework (PCF) classifies every process against the industry-standard process taxonomy (Cross-Industry plus industry variants) — a formal, provenance-linked capability/process reference. Coverage analytics then show which standard processes are modelled. Skills held by people and required by tasks read as ArchiMate Capabilities in the operating-model view.</t>
         </is>
@@ -8952,7 +8964,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diagramatix Miner monitors real value-stream performance from event logs, and the Simulator reports throughput/utilisation/flow-time. The organisation-wide Compliance Monitoring console additionally trends control operating-effectiveness over time across every project — with below-threshold and declining-control alerts — rolled up by APQC process category. Every mined figure declares its own exactness — whole run, this slice, or an estimate — and period comparison shows when the value stream changed.</t>
         </is>
@@ -8980,7 +8992,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G4" s="39" t="inlineStr">
+      <c r="G4" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">The Simulator and Diagramatix Miner both report how a process is performing (simulated and actual), and the org-wide Compliance Monitoring console adds continuous, over-time monitoring of control-effectiveness across all projects. Task Mining adds an Automation tab per task: automation score, ping-pong and rework detection, an RPA specification and ROI.</t>
         </is>
@@ -9152,7 +9164,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G10" s="39" t="inlineStr">
+      <c r="G10" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Simulation input data is created via simulation parameters and calendars, and Diagramatix Miner calibrates the inputs automatically from real event logs. Distribution fitting selects lognormal / empirical / triangular shapes from the observed values, and a mined calibration is tested on held-back cases the model never saw.</t>
         </is>
@@ -9283,7 +9295,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Multi-notation modelling supports Value Chain chevrons, BPMN collapsed sub-processes and ArchiMate Processes/Functions in one workspace. EPC (eEPC) is a tenth notation, with ARIS AML import and a deterministic Convert to BPMN.</t>
         </is>
@@ -9311,7 +9323,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G4" s="39" t="inlineStr">
+      <c r="G4" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">The Simulator and Diagramatix Miner identify bottlenecks and prove the redesign case for low-performing processes. The Simulator then defends the redesign: a significance test on the difference, a parameter sweep with the knee marked, a sensitivity tornado, validation against the actual flow-time distribution, and a business case with a payback month.</t>
         </is>
@@ -9362,17 +9374,17 @@
       <c r="E6" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="F6" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comply</t>
-        </is>
-      </c>
-      <c r="G6" s="39" t="inlineStr">
+      <c r="F6" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
+        </is>
+      </c>
+      <c r="G6" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Real-time co-authoring: every editor sees who else is in the diagram (presence and live cursors); an element being edited by someone else is soft-locked and shown as a ghost; and a version guard with automatic three-way merge means a concurrent save can never silently override another modeller's changes. Diagram history records who changed what.</t>
         </is>
       </c>
-      <c r="H6" s="39"/>
+      <c r="H6" s="43"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
@@ -9418,17 +9430,17 @@
       <c r="E8" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="F8" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comply</t>
-        </is>
-      </c>
-      <c r="G8" s="39" t="inlineStr">
+      <c r="F8" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
+        </is>
+      </c>
+      <c r="G8" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Live presence and cursors show the moment another user opens the diagram, their in-progress edits appear as live ghosts, and a save that would conflict is detected by the version guard and merged (or surfaced) rather than applied blind. Diagram history retains who changed what and when.</t>
         </is>
       </c>
-      <c r="H8" s="39"/>
+      <c r="H8" s="43"/>
     </row>
     <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
@@ -9594,17 +9606,17 @@
       <c r="E14" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="F14" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comply</t>
-        </is>
-      </c>
-      <c r="G14" s="39" t="inlineStr">
+      <c r="F14" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
+        </is>
+      </c>
+      <c r="G14" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Diff Processes compares two versions of a BPMN process (or two diagrams) — elements added, removed and renamed, flows changed, lane moves — as a table with CSV and Word (.docx) export and an AI narrative of the gap, kept in a per-project run history. The Simulator's as-is/to-be studies then quantify the operational difference.</t>
         </is>
       </c>
-      <c r="H14" s="39"/>
+      <c r="H14" s="43"/>
     </row>
     <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
@@ -9867,7 +9879,7 @@
           <t xml:space="preserve">Partially Comply</t>
         </is>
       </c>
-      <c r="G23" s="39" t="inlineStr">
+      <c r="G23" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Publishing produces versioned process documentation with a Title Block (version/authors/status), descriptions, hyperlinks to work instructions/business rules and embedded diagrams; bundles group related diagrams. SOP documents are generated to Word adopting the organisation's Word template, with a true-to-layout preview.</t>
         </is>
@@ -9931,7 +9943,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G25" s="39" t="inlineStr">
+      <c r="G25" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">AI Generate (text-to-diagram) and Voice Dictation create process outline diagrams instantly — a true rapid/quick modelling capability. “Create APQC Process” also generates a running BPMN model from a chosen standard APQC process in one click (higher-level processes decompose into collapsed sub-processes; task-level processes are AI-generated), so modellers can start straight from the recognised industry standard. Generation runs on the LLM the organisation chooses — seven providers, including a fully local model — with per-org cost metering; Abracadabra Mode applies spoken or typed edits live ('add a task after Review'), undoable and validated by the same rules engine.</t>
         </is>
@@ -10075,7 +10087,7 @@
           <t xml:space="preserve">Comply</t>
         </is>
       </c>
-      <c r="G30" s="39" t="inlineStr">
+      <c r="G30" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">The Simulator captures per-task execution cost and frequency (arrival/branch data), and Diagramatix Miner derives real frequencies and durations from event logs. Per-run activity charges (costs that do not scale with time) are captured separately from resource cost.</t>
         </is>

</xml_diff>